<commit_message>
Implementação da configuração para escolha de integração das despesas, e bug fix na verificação da importação dos documentos no domínio
</commit_message>
<xml_diff>
--- a/BateriasDeTestes/Teste-01.xlsx
+++ b/BateriasDeTestes/Teste-01.xlsx
@@ -3,11 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Teste-01" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Teste-02" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Folha1" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr/>
   <extLst>
@@ -17,7 +18,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+  <si>
+    <t xml:space="preserve">Empresa sem movimento</t>
+  </si>
   <si>
     <t xml:space="preserve">Erro na integração das despesas, favor verificar</t>
   </si>
@@ -614,6 +618,9 @@
       <c r="B9" s="1">
         <v>39450253000100</v>
       </c>
+      <c r="C9" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="10" ht="14.25">
       <c r="B10" s="1">
@@ -630,7 +637,7 @@
         <v>28460213000115</v>
       </c>
       <c r="C12" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" ht="14.25">
@@ -753,4 +760,99 @@
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col customWidth="1" min="2" max="2" width="27.421875"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1">
+        <v>42137437000111</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="1">
+        <v>42197710000101</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="1">
+        <v>42247681000137</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="1">
+        <v>42486567000160</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="1">
+        <v>42816024000163</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="1">
+        <v>42952963000135</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="1">
+        <v>44209825000196</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="1">
+        <v>44787128000112</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="1">
+        <v>45228365000106</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="1">
+        <v>45916615000109</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="1">
+        <v>45929899000160</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="1">
+        <v>45942890000199</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="1">
+        <v>46014135000107</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="1">
+        <v>46752607000129</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="1">
+        <v>47020716000114</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="1">
+        <v>47151060000179</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>